<commit_message>
add: Correcion retenciones emitidas.
</commit_message>
<xml_diff>
--- a/api/src/main/resources/importaciones/rrhh-novedades.xlsx
+++ b/api/src/main/resources/importaciones/rrhh-novedades.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ismael\Documents\calero-app-desktop\api\src\main\resources\importaciones\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB8019E2-A292-4A99-96E0-D5E0D0B250DB}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD24BBD8-C79E-426A-9D30-1DDB17E362CF}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="22">
   <si>
     <t>AÑO</t>
   </si>
@@ -58,31 +58,34 @@
     <t>Sobresueldos, comisiones y otras remuneraciones gravadas de I.Renta (materia NO gravada de seguridad social)</t>
   </si>
   <si>
-    <t>1790715949001</t>
-  </si>
-  <si>
-    <t>0190151530001</t>
-  </si>
-  <si>
-    <t>0300855368001</t>
-  </si>
-  <si>
-    <t>1760000740001</t>
-  </si>
-  <si>
-    <t>1760003410001</t>
-  </si>
-  <si>
-    <t>1791131606001</t>
-  </si>
-  <si>
-    <t>1751136138001</t>
-  </si>
-  <si>
-    <t>1751126138001</t>
-  </si>
-  <si>
-    <t>1751134138001</t>
+    <t>1234567891001</t>
+  </si>
+  <si>
+    <t>1234567892001</t>
+  </si>
+  <si>
+    <t>1234567893001</t>
+  </si>
+  <si>
+    <t>1234567894001</t>
+  </si>
+  <si>
+    <t>1234567895001</t>
+  </si>
+  <si>
+    <t>1234567896001</t>
+  </si>
+  <si>
+    <t>1234567897001</t>
+  </si>
+  <si>
+    <t>1234567898001</t>
+  </si>
+  <si>
+    <t>1234567899001</t>
+  </si>
+  <si>
+    <t>2026-12</t>
   </si>
 </sst>
 </file>
@@ -581,7 +584,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:M11"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.5703125" style="3"/>
@@ -637,8 +640,8 @@
       </c>
     </row>
     <row r="2" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="4">
-        <v>2023</v>
+      <c r="A2" s="3" t="s">
+        <v>21</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>12</v>
@@ -676,8 +679,8 @@
       <c r="M2" s="5"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A3" s="4">
-        <v>2023</v>
+      <c r="A3" s="3" t="s">
+        <v>21</v>
       </c>
       <c r="B3" s="7" t="s">
         <v>13</v>
@@ -713,11 +716,11 @@
       <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A4" s="4">
-        <v>2023</v>
+      <c r="A4" s="3" t="s">
+        <v>21</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C4" s="1">
         <v>1400</v>
@@ -750,51 +753,73 @@
       <c r="M4" s="1"/>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A5" s="4"/>
-      <c r="B5" s="7"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
+      <c r="A5" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="1">
+        <v>2200</v>
+      </c>
+      <c r="D5" s="1">
+        <v>0</v>
+      </c>
       <c r="E5" s="1"/>
-      <c r="F5" s="1"/>
-      <c r="G5" s="1"/>
-      <c r="H5" s="2"/>
-      <c r="I5" s="1"/>
-      <c r="J5" s="1"/>
-      <c r="K5" s="1"/>
-      <c r="L5" s="1"/>
+      <c r="F5" s="1">
+        <v>43.92</v>
+      </c>
+      <c r="G5" s="1">
+        <v>169.98</v>
+      </c>
+      <c r="H5" s="2">
+        <v>43.9</v>
+      </c>
+      <c r="I5" s="1">
+        <v>0</v>
+      </c>
+      <c r="J5" s="1">
+        <v>671.22</v>
+      </c>
+      <c r="K5" s="1">
+        <v>600</v>
+      </c>
+      <c r="L5" s="1">
+        <v>0</v>
+      </c>
       <c r="M5" s="1"/>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A6" s="4">
-        <v>2023</v>
+      <c r="A6" s="3" t="s">
+        <v>21</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C6" s="1">
-        <v>2200</v>
+        <v>3000</v>
       </c>
       <c r="D6" s="1">
         <v>0</v>
       </c>
       <c r="E6" s="1"/>
       <c r="F6" s="1">
-        <v>43.92</v>
+        <v>3559.49</v>
       </c>
       <c r="G6" s="1">
-        <v>169.98</v>
+        <v>340</v>
       </c>
       <c r="H6" s="2">
-        <v>43.9</v>
+        <v>2862.65</v>
       </c>
       <c r="I6" s="1">
         <v>0</v>
       </c>
       <c r="J6" s="1">
-        <v>671.22</v>
+        <v>0</v>
       </c>
       <c r="K6" s="1">
-        <v>600</v>
+        <v>700</v>
       </c>
       <c r="L6" s="1">
         <v>0</v>
@@ -802,27 +827,27 @@
       <c r="M6" s="1"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A7" s="4">
-        <v>2023</v>
+      <c r="A7" s="3" t="s">
+        <v>21</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C7" s="1">
-        <v>3000</v>
+        <v>5000</v>
       </c>
       <c r="D7" s="1">
-        <v>0</v>
+        <v>342.07</v>
       </c>
       <c r="E7" s="1"/>
       <c r="F7" s="1">
-        <v>3559.49</v>
+        <v>578.26</v>
       </c>
       <c r="G7" s="1">
-        <v>340</v>
-      </c>
-      <c r="H7" s="2">
-        <v>2862.65</v>
+        <v>125.43</v>
+      </c>
+      <c r="H7" s="1">
+        <v>0</v>
       </c>
       <c r="I7" s="1">
         <v>0</v>
@@ -831,7 +856,7 @@
         <v>0</v>
       </c>
       <c r="K7" s="1">
-        <v>700</v>
+        <v>750</v>
       </c>
       <c r="L7" s="1">
         <v>0</v>
@@ -839,24 +864,24 @@
       <c r="M7" s="1"/>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A8" s="4">
-        <v>2023</v>
+      <c r="A8" s="3" t="s">
+        <v>21</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C8" s="1">
-        <v>5000</v>
+        <v>6000</v>
       </c>
       <c r="D8" s="1">
-        <v>342.07</v>
+        <v>0</v>
       </c>
       <c r="E8" s="1"/>
       <c r="F8" s="1">
-        <v>578.26</v>
+        <v>505</v>
       </c>
       <c r="G8" s="1">
-        <v>125.43</v>
+        <v>79.5</v>
       </c>
       <c r="H8" s="1">
         <v>0</v>
@@ -865,10 +890,10 @@
         <v>0</v>
       </c>
       <c r="J8" s="1">
-        <v>0</v>
+        <v>1074.6400000000001</v>
       </c>
       <c r="K8" s="1">
-        <v>750</v>
+        <v>900</v>
       </c>
       <c r="L8" s="1">
         <v>0</v>
@@ -876,24 +901,24 @@
       <c r="M8" s="1"/>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A9" s="4">
-        <v>2023</v>
+      <c r="A9" s="3" t="s">
+        <v>21</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C9" s="1">
-        <v>6000</v>
+        <v>12000</v>
       </c>
       <c r="D9" s="1">
         <v>0</v>
       </c>
       <c r="E9" s="1"/>
       <c r="F9" s="1">
-        <v>505</v>
+        <v>48.75</v>
       </c>
       <c r="G9" s="1">
-        <v>79.5</v>
+        <v>26.5</v>
       </c>
       <c r="H9" s="1">
         <v>0</v>
@@ -902,10 +927,10 @@
         <v>0</v>
       </c>
       <c r="J9" s="1">
-        <v>1074.6400000000001</v>
+        <v>47.19</v>
       </c>
       <c r="K9" s="1">
-        <v>900</v>
+        <v>2000</v>
       </c>
       <c r="L9" s="1">
         <v>0</v>
@@ -913,24 +938,24 @@
       <c r="M9" s="1"/>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A10" s="4">
-        <v>2023</v>
+      <c r="A10" s="3" t="s">
+        <v>21</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C10" s="1">
-        <v>12000</v>
+        <v>15000</v>
       </c>
       <c r="D10" s="1">
-        <v>0</v>
+        <v>443.68</v>
       </c>
       <c r="E10" s="1"/>
       <c r="F10" s="1">
-        <v>48.75</v>
+        <v>178.47</v>
       </c>
       <c r="G10" s="1">
-        <v>26.5</v>
+        <v>0</v>
       </c>
       <c r="H10" s="1">
         <v>0</v>
@@ -939,52 +964,15 @@
         <v>0</v>
       </c>
       <c r="J10" s="1">
-        <v>47.19</v>
+        <v>0</v>
       </c>
       <c r="K10" s="1">
-        <v>2000</v>
+        <v>3500</v>
       </c>
       <c r="L10" s="1">
         <v>0</v>
       </c>
       <c r="M10" s="1"/>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A11" s="4">
-        <v>2023</v>
-      </c>
-      <c r="B11" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="C11" s="1">
-        <v>15000</v>
-      </c>
-      <c r="D11" s="1">
-        <v>443.68</v>
-      </c>
-      <c r="E11" s="1"/>
-      <c r="F11" s="1">
-        <v>178.47</v>
-      </c>
-      <c r="G11" s="1">
-        <v>0</v>
-      </c>
-      <c r="H11" s="1">
-        <v>0</v>
-      </c>
-      <c r="I11" s="1">
-        <v>0</v>
-      </c>
-      <c r="J11" s="1">
-        <v>0</v>
-      </c>
-      <c r="K11" s="1">
-        <v>3500</v>
-      </c>
-      <c r="L11" s="1">
-        <v>0</v>
-      </c>
-      <c r="M11" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>